<commit_message>
Fixed: PORT Field Accepts Lowercase Values
</commit_message>
<xml_diff>
--- a/uploads/items.xlsx
+++ b/uploads/items.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
   <si>
     <t>NO. OF PACKAGE</t>
   </si>
@@ -167,10 +167,13 @@
     <t>CONTAINER SIZE</t>
   </si>
   <si>
+    <t>APPLETON GRP LLC</t>
+  </si>
+  <si>
     <t>C/O KWE-Kintetsu World Express (S) Pte Ltd. 20 Changi South Avenue 2 Singapore 486547</t>
   </si>
   <si>
-    <t>APPLETON GRP LLC-_.,:;#$%()*/</t>
+    <t>p03</t>
   </si>
 </sst>
 </file>
@@ -653,13 +656,13 @@
     </row>
     <row r="2" spans="1:12" s="2" customFormat="1">
       <c r="A2" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>46</v>
-      </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Fix: COUNTRY OF DESTINATION, PORT OF LOADING, and PORT OF DEPARTURE fields Accept Lowercase Input
</commit_message>
<xml_diff>
--- a/uploads/items.xlsx
+++ b/uploads/items.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
   <si>
     <t>NO. OF PACKAGE</t>
   </si>
@@ -137,6 +137,9 @@
     <t>TESTING</t>
   </si>
   <si>
+    <t>A17</t>
+  </si>
+  <si>
     <t>PORT OF DEPARTURE</t>
   </si>
   <si>
@@ -146,12 +149,6 @@
     <t>SEAL NUMBER</t>
   </si>
   <si>
-    <t>JP</t>
-  </si>
-  <si>
-    <t>PHABU</t>
-  </si>
-  <si>
     <t>B20260017</t>
   </si>
   <si>
@@ -170,14 +167,20 @@
     <t>C/O KWE-Kintetsu World Express (S) Pte Ltd. 20 Changi South Avenue 2 Singapore 486547</t>
   </si>
   <si>
-    <t>a17</t>
+    <t>p03</t>
+  </si>
+  <si>
+    <t>ph</t>
+  </si>
+  <si>
+    <t>phabu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +202,12 @@
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -228,7 +237,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -236,11 +245,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -263,6 +287,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -613,7 +640,7 @@
     <col min="11" max="12" width="24.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="14.5" thickBot="1">
       <c r="A1" s="6" t="s">
         <v>29</v>
       </c>
@@ -645,18 +672,18 @@
         <v>24</v>
       </c>
       <c r="K1" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="L1" s="6" t="s">
-        <v>36</v>
-      </c>
     </row>
-    <row r="2" spans="1:12" s="2" customFormat="1">
+    <row r="2" spans="1:12" s="2" customFormat="1" ht="14.5" thickBot="1">
       <c r="A2" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>45</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>46</v>
       </c>
       <c r="C2" t="s">
         <v>33</v>
@@ -674,19 +701,19 @@
         <v>35</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="I2" s="2">
         <v>140100000</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>33</v>
+      <c r="J2" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="9" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -710,10 +737,10 @@
         <v>14</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -775,7 +802,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -808,7 +835,7 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -841,7 +868,7 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Fix: NO. OF PACKAGE Field Allows Invalid Zero and Empty Values
</commit_message>
<xml_diff>
--- a/uploads/items.xlsx
+++ b/uploads/items.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10700"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10700" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
   <si>
     <t>NO. OF PACKAGE</t>
   </si>
@@ -149,6 +149,12 @@
     <t>SEAL NUMBER</t>
   </si>
   <si>
+    <t>JP</t>
+  </si>
+  <si>
+    <t>PHABU</t>
+  </si>
+  <si>
     <t>B20260017</t>
   </si>
   <si>
@@ -165,22 +171,13 @@
   </si>
   <si>
     <t>C/O KWE-Kintetsu World Express (S) Pte Ltd. 20 Changi South Avenue 2 Singapore 486547</t>
-  </si>
-  <si>
-    <t>p03</t>
-  </si>
-  <si>
-    <t>ph</t>
-  </si>
-  <si>
-    <t>phabu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,12 +199,6 @@
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -237,7 +228,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -245,26 +236,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -287,9 +263,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -640,7 +613,7 @@
     <col min="11" max="12" width="24.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" ht="14.5" thickBot="1">
+    <row r="1" spans="1:12" s="1" customFormat="1">
       <c r="A1" s="6" t="s">
         <v>29</v>
       </c>
@@ -678,12 +651,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="2" customFormat="1" ht="14.5" thickBot="1">
+    <row r="2" spans="1:12" s="2" customFormat="1">
       <c r="A2" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
         <v>33</v>
@@ -706,14 +679,14 @@
       <c r="I2" s="2">
         <v>140100000</v>
       </c>
-      <c r="J2" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="L2" s="9" t="s">
-        <v>46</v>
+      <c r="J2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -740,7 +713,7 @@
         <v>39</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -802,13 +775,13 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -835,14 +808,12 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2">
-        <v>0</v>
-      </c>
+      <c r="C3" s="2"/>
       <c r="D3" t="s">
         <v>12</v>
       </c>
@@ -868,7 +839,7 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Fix: CONTAINER NUMBER and SEAL NUMBER Fields
</commit_message>
<xml_diff>
--- a/uploads/items.xlsx
+++ b/uploads/items.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10700" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10700" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="55">
   <si>
     <t>NO. OF PACKAGE</t>
   </si>
@@ -110,6 +110,9 @@
     <t>Terms of Payment</t>
   </si>
   <si>
+    <t>FOB</t>
+  </si>
+  <si>
     <t>01</t>
   </si>
   <si>
@@ -188,7 +191,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>fob</t>
+    <t>MSKU1234567</t>
   </si>
 </sst>
 </file>
@@ -279,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -324,6 +327,12 @@
     </xf>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -676,16 +685,16 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1">
       <c r="A1" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>18</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>19</v>
@@ -706,48 +715,48 @@
         <v>24</v>
       </c>
       <c r="K1" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:12" s="2" customFormat="1">
       <c r="A2" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F2" s="2">
         <v>1234567891</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I2" s="2">
         <v>140100000</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -758,23 +767,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:3" ht="14.5" thickBot="1">
+      <c r="A1" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>44</v>
+      <c r="B1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="14.5" thickBot="1">
+      <c r="A2" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -836,7 +853,7 @@
     </row>
     <row r="2" spans="1:11" ht="14.5" thickBot="1">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -858,18 +875,18 @@
         <v>17</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="14.5" thickBot="1">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -891,18 +908,18 @@
         <v>17</v>
       </c>
       <c r="I3" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="16" t="s">
         <v>49</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="K3" s="16" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="14.5" thickBot="1">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -928,7 +945,7 @@
       <c r="I4" s="15"/>
       <c r="J4" s="15"/>
       <c r="K4" s="14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -956,10 +973,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>